<commit_message>
commiting before starting new branch
</commit_message>
<xml_diff>
--- a/extensive_test/test_schedule_output.xlsx
+++ b/extensive_test/test_schedule_output.xlsx
@@ -46,7 +46,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE68A"/>
+        <fgColor rgb="00FCA5A5"/>
       </patternFill>
     </fill>
     <fill>
@@ -56,17 +56,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCA5A5"/>
+        <fgColor rgb="00FCD34D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0093C5FD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCD34D"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,10 +109,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -607,92 +607,92 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
+          <t>Frank Miller</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Eli Jones</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Oliver Moore</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Daniel Hernandez</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Zack Walker</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
           <t>Chloe Young</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Aaron Smith</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Kevin Martinez</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Liam Anderson</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Oliver Moore</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Henry Garcia</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Rodriguez</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>David Brown</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Caleb Williams</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Oliver Moore</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Jack Wilson</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Alice Hall</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Tom Thompson</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Jack Wilson</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>David Brown</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>Noah Thomas</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Quinn Martin</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>Xavier Lewis</t>
-        </is>
-      </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>Noah Thomas</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>Caleb Williams</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>Yara Robinson</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>David Brown</t>
-        </is>
-      </c>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>Henry Garcia</t>
-        </is>
-      </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>Jack Wilson</t>
-        </is>
-      </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>Ben Johnson</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
         <is>
           <t>Liam Anderson</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
-        <is>
-          <t>Isaac Rodriguez</t>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>Paul Jackson</t>
         </is>
       </c>
     </row>
@@ -702,94 +702,94 @@
           <t>Gate Guard 2</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Daniel Hernandez</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>George Davis</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>David Brown</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Rodriguez</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Tom Thompson</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Paul Jackson</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Ben Johnson</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Tom Thompson</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Chloe Young</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Sarah Perez</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>George Davis</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Isaac Rodriguez</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Aaron Smith</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Frank Miller</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Jack Wilson</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Mason Taylor</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Eli Jones</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Noah Thomas</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Kevin Martinez</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Henry Garcia</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>Caleb Williams</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>George Davis</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Sarah Perez</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>David Brown</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>Henry Garcia</t>
-        </is>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>Mason Taylor</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>Aaron Smith</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>Noah Thomas</t>
-        </is>
-      </c>
-      <c r="Q3" s="6" t="inlineStr">
-        <is>
-          <t>Quinn Martin</t>
-        </is>
-      </c>
-      <c r="R3" s="4" t="inlineStr">
-        <is>
-          <t>Caleb Williams</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>George Davis</t>
         </is>
       </c>
     </row>
@@ -877,49 +877,49 @@
           <t>HQ Duty</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Quinn Martin</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Mason Taylor</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Sarah Perez</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Rodriguez</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Aaron Smith</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Caleb Williams</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Eli Jones</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Zack Walker</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Paul Jackson</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Ben Johnson</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Xavier Lewis</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Zack Walker</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Tom Thompson</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Sarah Perez</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>Xavier Lewis</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Isaac Rodriguez</t>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>George Davis</t>
         </is>
       </c>
     </row>
@@ -1009,21 +1009,21 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Alice Hall</t>
+          <t>Henry Garcia</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr"/>
       <c r="D2" s="8" t="inlineStr"/>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Sarah Perez</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Jack Wilson</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr"/>
       <c r="G2" s="8" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Paul Jackson</t>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Ursula White</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr"/>
@@ -1036,23 +1036,23 @@
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Paul Jackson</t>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Ursula White</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr"/>
       <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Paul Jackson</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Isaac Rodriguez</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr"/>
       <c r="H3" s="8" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>George Davis</t>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Sarah Perez</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr"/>
@@ -1067,21 +1067,21 @@
       <c r="C4" s="8" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Zack Walker</t>
+          <t>Jack Wilson</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr"/>
       <c r="F4" s="8" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Jack Wilson</t>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Quinn Martin</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr"/>
       <c r="I4" s="8" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Victor Harris</t>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>David Brown</t>
         </is>
       </c>
     </row>
@@ -1169,49 +1169,49 @@
           <t>Perimeter Patrol</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Kevin Martinez</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Xavier Lewis</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>Quinn Martin</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Isaac Rodriguez</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>Mason Taylor</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>David Brown</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Ben Johnson</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Eli Jones</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Xavier Lewis</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Oliver Moore</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>Liam Anderson</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Paul Jackson</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Frank Miller</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Henry Garcia</t>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Tom Thompson</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Sarah Perez</t>
         </is>
       </c>
     </row>
@@ -1281,32 +1281,32 @@
           <t>Standby Team A</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Eli Jones</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Ben Johnson</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Noah Thomas</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Victor Harris</t>
         </is>
       </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Ursula White</t>
+        </is>
+      </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Kevin Martinez</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Zack Walker</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
+          <t>Yara Robinson</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Quinn Martin</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Wendy Clark</t>
         </is>
@@ -1318,34 +1318,34 @@
           <t>Standby Team B</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Mason Taylor</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Bob Allen</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Aaron Smith</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Rachel Lee</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Bob Allen</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Yara Robinson</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Daniel Hernandez</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Chloe Young</t>
+          <t>Frank Miller</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Ursula White</t>
+          <t>Alice Hall</t>
         </is>
       </c>
     </row>

</xml_diff>